<commit_message>
Complete restoration of all UI components
</commit_message>
<xml_diff>
--- a/RTE_Status_Results.xlsx
+++ b/RTE_Status_Results.xlsx
@@ -625,7 +625,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>9054003184.0</t>
+          <t>9054003184</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>395003.0</t>
+          <t>395003</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">

</xml_diff>